<commit_message>
prise en compte des tags
</commit_message>
<xml_diff>
--- a/planning_output.xlsx
+++ b/planning_output.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:GT26"/>
+  <dimension ref="A1:MR14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -648,6 +648,160 @@
     <col width="8" customWidth="1" min="200" max="200"/>
     <col width="8" customWidth="1" min="201" max="201"/>
     <col width="8" customWidth="1" min="202" max="202"/>
+    <col width="8" customWidth="1" min="203" max="203"/>
+    <col width="8" customWidth="1" min="204" max="204"/>
+    <col width="8" customWidth="1" min="205" max="205"/>
+    <col width="8" customWidth="1" min="206" max="206"/>
+    <col width="8" customWidth="1" min="207" max="207"/>
+    <col width="8" customWidth="1" min="208" max="208"/>
+    <col width="8" customWidth="1" min="209" max="209"/>
+    <col width="8" customWidth="1" min="210" max="210"/>
+    <col width="8" customWidth="1" min="211" max="211"/>
+    <col width="8" customWidth="1" min="212" max="212"/>
+    <col width="8" customWidth="1" min="213" max="213"/>
+    <col width="8" customWidth="1" min="214" max="214"/>
+    <col width="8" customWidth="1" min="215" max="215"/>
+    <col width="8" customWidth="1" min="216" max="216"/>
+    <col width="8" customWidth="1" min="217" max="217"/>
+    <col width="8" customWidth="1" min="218" max="218"/>
+    <col width="8" customWidth="1" min="219" max="219"/>
+    <col width="8" customWidth="1" min="220" max="220"/>
+    <col width="8" customWidth="1" min="221" max="221"/>
+    <col width="8" customWidth="1" min="222" max="222"/>
+    <col width="8" customWidth="1" min="223" max="223"/>
+    <col width="8" customWidth="1" min="224" max="224"/>
+    <col width="8" customWidth="1" min="225" max="225"/>
+    <col width="8" customWidth="1" min="226" max="226"/>
+    <col width="8" customWidth="1" min="227" max="227"/>
+    <col width="8" customWidth="1" min="228" max="228"/>
+    <col width="8" customWidth="1" min="229" max="229"/>
+    <col width="8" customWidth="1" min="230" max="230"/>
+    <col width="8" customWidth="1" min="231" max="231"/>
+    <col width="8" customWidth="1" min="232" max="232"/>
+    <col width="8" customWidth="1" min="233" max="233"/>
+    <col width="8" customWidth="1" min="234" max="234"/>
+    <col width="8" customWidth="1" min="235" max="235"/>
+    <col width="8" customWidth="1" min="236" max="236"/>
+    <col width="8" customWidth="1" min="237" max="237"/>
+    <col width="8" customWidth="1" min="238" max="238"/>
+    <col width="8" customWidth="1" min="239" max="239"/>
+    <col width="8" customWidth="1" min="240" max="240"/>
+    <col width="8" customWidth="1" min="241" max="241"/>
+    <col width="8" customWidth="1" min="242" max="242"/>
+    <col width="8" customWidth="1" min="243" max="243"/>
+    <col width="8" customWidth="1" min="244" max="244"/>
+    <col width="8" customWidth="1" min="245" max="245"/>
+    <col width="8" customWidth="1" min="246" max="246"/>
+    <col width="8" customWidth="1" min="247" max="247"/>
+    <col width="8" customWidth="1" min="248" max="248"/>
+    <col width="8" customWidth="1" min="249" max="249"/>
+    <col width="8" customWidth="1" min="250" max="250"/>
+    <col width="8" customWidth="1" min="251" max="251"/>
+    <col width="8" customWidth="1" min="252" max="252"/>
+    <col width="8" customWidth="1" min="253" max="253"/>
+    <col width="8" customWidth="1" min="254" max="254"/>
+    <col width="8" customWidth="1" min="255" max="255"/>
+    <col width="8" customWidth="1" min="256" max="256"/>
+    <col width="8" customWidth="1" min="257" max="257"/>
+    <col width="8" customWidth="1" min="258" max="258"/>
+    <col width="8" customWidth="1" min="259" max="259"/>
+    <col width="8" customWidth="1" min="260" max="260"/>
+    <col width="8" customWidth="1" min="261" max="261"/>
+    <col width="8" customWidth="1" min="262" max="262"/>
+    <col width="8" customWidth="1" min="263" max="263"/>
+    <col width="8" customWidth="1" min="264" max="264"/>
+    <col width="8" customWidth="1" min="265" max="265"/>
+    <col width="8" customWidth="1" min="266" max="266"/>
+    <col width="8" customWidth="1" min="267" max="267"/>
+    <col width="8" customWidth="1" min="268" max="268"/>
+    <col width="8" customWidth="1" min="269" max="269"/>
+    <col width="8" customWidth="1" min="270" max="270"/>
+    <col width="8" customWidth="1" min="271" max="271"/>
+    <col width="8" customWidth="1" min="272" max="272"/>
+    <col width="8" customWidth="1" min="273" max="273"/>
+    <col width="8" customWidth="1" min="274" max="274"/>
+    <col width="8" customWidth="1" min="275" max="275"/>
+    <col width="8" customWidth="1" min="276" max="276"/>
+    <col width="8" customWidth="1" min="277" max="277"/>
+    <col width="8" customWidth="1" min="278" max="278"/>
+    <col width="8" customWidth="1" min="279" max="279"/>
+    <col width="8" customWidth="1" min="280" max="280"/>
+    <col width="8" customWidth="1" min="281" max="281"/>
+    <col width="8" customWidth="1" min="282" max="282"/>
+    <col width="8" customWidth="1" min="283" max="283"/>
+    <col width="8" customWidth="1" min="284" max="284"/>
+    <col width="8" customWidth="1" min="285" max="285"/>
+    <col width="8" customWidth="1" min="286" max="286"/>
+    <col width="8" customWidth="1" min="287" max="287"/>
+    <col width="8" customWidth="1" min="288" max="288"/>
+    <col width="8" customWidth="1" min="289" max="289"/>
+    <col width="8" customWidth="1" min="290" max="290"/>
+    <col width="8" customWidth="1" min="291" max="291"/>
+    <col width="8" customWidth="1" min="292" max="292"/>
+    <col width="8" customWidth="1" min="293" max="293"/>
+    <col width="8" customWidth="1" min="294" max="294"/>
+    <col width="8" customWidth="1" min="295" max="295"/>
+    <col width="8" customWidth="1" min="296" max="296"/>
+    <col width="8" customWidth="1" min="297" max="297"/>
+    <col width="8" customWidth="1" min="298" max="298"/>
+    <col width="8" customWidth="1" min="299" max="299"/>
+    <col width="8" customWidth="1" min="300" max="300"/>
+    <col width="8" customWidth="1" min="301" max="301"/>
+    <col width="8" customWidth="1" min="302" max="302"/>
+    <col width="8" customWidth="1" min="303" max="303"/>
+    <col width="8" customWidth="1" min="304" max="304"/>
+    <col width="8" customWidth="1" min="305" max="305"/>
+    <col width="8" customWidth="1" min="306" max="306"/>
+    <col width="8" customWidth="1" min="307" max="307"/>
+    <col width="8" customWidth="1" min="308" max="308"/>
+    <col width="8" customWidth="1" min="309" max="309"/>
+    <col width="8" customWidth="1" min="310" max="310"/>
+    <col width="8" customWidth="1" min="311" max="311"/>
+    <col width="8" customWidth="1" min="312" max="312"/>
+    <col width="8" customWidth="1" min="313" max="313"/>
+    <col width="8" customWidth="1" min="314" max="314"/>
+    <col width="8" customWidth="1" min="315" max="315"/>
+    <col width="8" customWidth="1" min="316" max="316"/>
+    <col width="8" customWidth="1" min="317" max="317"/>
+    <col width="8" customWidth="1" min="318" max="318"/>
+    <col width="8" customWidth="1" min="319" max="319"/>
+    <col width="8" customWidth="1" min="320" max="320"/>
+    <col width="8" customWidth="1" min="321" max="321"/>
+    <col width="8" customWidth="1" min="322" max="322"/>
+    <col width="8" customWidth="1" min="323" max="323"/>
+    <col width="8" customWidth="1" min="324" max="324"/>
+    <col width="8" customWidth="1" min="325" max="325"/>
+    <col width="8" customWidth="1" min="326" max="326"/>
+    <col width="8" customWidth="1" min="327" max="327"/>
+    <col width="8" customWidth="1" min="328" max="328"/>
+    <col width="8" customWidth="1" min="329" max="329"/>
+    <col width="8" customWidth="1" min="330" max="330"/>
+    <col width="8" customWidth="1" min="331" max="331"/>
+    <col width="8" customWidth="1" min="332" max="332"/>
+    <col width="8" customWidth="1" min="333" max="333"/>
+    <col width="8" customWidth="1" min="334" max="334"/>
+    <col width="8" customWidth="1" min="335" max="335"/>
+    <col width="8" customWidth="1" min="336" max="336"/>
+    <col width="8" customWidth="1" min="337" max="337"/>
+    <col width="8" customWidth="1" min="338" max="338"/>
+    <col width="8" customWidth="1" min="339" max="339"/>
+    <col width="8" customWidth="1" min="340" max="340"/>
+    <col width="8" customWidth="1" min="341" max="341"/>
+    <col width="8" customWidth="1" min="342" max="342"/>
+    <col width="8" customWidth="1" min="343" max="343"/>
+    <col width="8" customWidth="1" min="344" max="344"/>
+    <col width="8" customWidth="1" min="345" max="345"/>
+    <col width="8" customWidth="1" min="346" max="346"/>
+    <col width="8" customWidth="1" min="347" max="347"/>
+    <col width="8" customWidth="1" min="348" max="348"/>
+    <col width="8" customWidth="1" min="349" max="349"/>
+    <col width="8" customWidth="1" min="350" max="350"/>
+    <col width="8" customWidth="1" min="351" max="351"/>
+    <col width="8" customWidth="1" min="352" max="352"/>
+    <col width="8" customWidth="1" min="353" max="353"/>
+    <col width="8" customWidth="1" min="354" max="354"/>
+    <col width="8" customWidth="1" min="355" max="355"/>
+    <col width="8" customWidth="1" min="356" max="356"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -841,7 +995,11 @@
       <c r="FX1" s="1" t="n"/>
       <c r="FY1" s="1" t="n"/>
       <c r="FZ1" s="1" t="n"/>
-      <c r="GA1" s="1" t="n"/>
+      <c r="GA1" s="1" t="inlineStr">
+        <is>
+          <t>March 2026</t>
+        </is>
+      </c>
       <c r="GB1" s="1" t="n"/>
       <c r="GC1" s="1" t="n"/>
       <c r="GD1" s="1" t="n"/>
@@ -861,6 +1019,160 @@
       <c r="GR1" s="1" t="n"/>
       <c r="GS1" s="1" t="n"/>
       <c r="GT1" s="1" t="n"/>
+      <c r="GU1" s="1" t="n"/>
+      <c r="GV1" s="1" t="n"/>
+      <c r="GW1" s="1" t="n"/>
+      <c r="GX1" s="1" t="n"/>
+      <c r="GY1" s="1" t="n"/>
+      <c r="GZ1" s="1" t="n"/>
+      <c r="HA1" s="1" t="n"/>
+      <c r="HB1" s="1" t="n"/>
+      <c r="HC1" s="1" t="n"/>
+      <c r="HD1" s="1" t="n"/>
+      <c r="HE1" s="1" t="n"/>
+      <c r="HF1" s="1" t="n"/>
+      <c r="HG1" s="1" t="n"/>
+      <c r="HH1" s="1" t="n"/>
+      <c r="HI1" s="1" t="n"/>
+      <c r="HJ1" s="1" t="n"/>
+      <c r="HK1" s="1" t="n"/>
+      <c r="HL1" s="1" t="n"/>
+      <c r="HM1" s="1" t="n"/>
+      <c r="HN1" s="1" t="n"/>
+      <c r="HO1" s="1" t="n"/>
+      <c r="HP1" s="1" t="n"/>
+      <c r="HQ1" s="1" t="n"/>
+      <c r="HR1" s="1" t="n"/>
+      <c r="HS1" s="1" t="n"/>
+      <c r="HT1" s="1" t="n"/>
+      <c r="HU1" s="1" t="n"/>
+      <c r="HV1" s="1" t="n"/>
+      <c r="HW1" s="1" t="n"/>
+      <c r="HX1" s="1" t="n"/>
+      <c r="HY1" s="1" t="n"/>
+      <c r="HZ1" s="1" t="n"/>
+      <c r="IA1" s="1" t="n"/>
+      <c r="IB1" s="1" t="n"/>
+      <c r="IC1" s="1" t="n"/>
+      <c r="ID1" s="1" t="n"/>
+      <c r="IE1" s="1" t="n"/>
+      <c r="IF1" s="1" t="n"/>
+      <c r="IG1" s="1" t="n"/>
+      <c r="IH1" s="1" t="n"/>
+      <c r="II1" s="1" t="n"/>
+      <c r="IJ1" s="1" t="n"/>
+      <c r="IK1" s="1" t="n"/>
+      <c r="IL1" s="1" t="n"/>
+      <c r="IM1" s="1" t="n"/>
+      <c r="IN1" s="1" t="n"/>
+      <c r="IO1" s="1" t="n"/>
+      <c r="IP1" s="1" t="n"/>
+      <c r="IQ1" s="1" t="n"/>
+      <c r="IR1" s="1" t="n"/>
+      <c r="IS1" s="1" t="n"/>
+      <c r="IT1" s="1" t="n"/>
+      <c r="IU1" s="1" t="n"/>
+      <c r="IV1" s="1" t="n"/>
+      <c r="IW1" s="1" t="n"/>
+      <c r="IX1" s="1" t="n"/>
+      <c r="IY1" s="1" t="n"/>
+      <c r="IZ1" s="1" t="n"/>
+      <c r="JA1" s="1" t="n"/>
+      <c r="JB1" s="1" t="n"/>
+      <c r="JC1" s="1" t="n"/>
+      <c r="JD1" s="1" t="n"/>
+      <c r="JE1" s="1" t="n"/>
+      <c r="JF1" s="1" t="n"/>
+      <c r="JG1" s="1" t="n"/>
+      <c r="JH1" s="1" t="n"/>
+      <c r="JI1" s="1" t="n"/>
+      <c r="JJ1" s="1" t="n"/>
+      <c r="JK1" s="1" t="n"/>
+      <c r="JL1" s="1" t="n"/>
+      <c r="JM1" s="1" t="n"/>
+      <c r="JN1" s="1" t="n"/>
+      <c r="JO1" s="1" t="n"/>
+      <c r="JP1" s="1" t="n"/>
+      <c r="JQ1" s="1" t="n"/>
+      <c r="JR1" s="1" t="n"/>
+      <c r="JS1" s="1" t="n"/>
+      <c r="JT1" s="1" t="n"/>
+      <c r="JU1" s="1" t="n"/>
+      <c r="JV1" s="1" t="n"/>
+      <c r="JW1" s="1" t="n"/>
+      <c r="JX1" s="1" t="n"/>
+      <c r="JY1" s="1" t="n"/>
+      <c r="JZ1" s="1" t="n"/>
+      <c r="KA1" s="1" t="n"/>
+      <c r="KB1" s="1" t="n"/>
+      <c r="KC1" s="1" t="n"/>
+      <c r="KD1" s="1" t="n"/>
+      <c r="KE1" s="1" t="n"/>
+      <c r="KF1" s="1" t="n"/>
+      <c r="KG1" s="1" t="n"/>
+      <c r="KH1" s="1" t="n"/>
+      <c r="KI1" s="1" t="n"/>
+      <c r="KJ1" s="1" t="n"/>
+      <c r="KK1" s="1" t="n"/>
+      <c r="KL1" s="1" t="n"/>
+      <c r="KM1" s="1" t="n"/>
+      <c r="KN1" s="1" t="n"/>
+      <c r="KO1" s="1" t="n"/>
+      <c r="KP1" s="1" t="n"/>
+      <c r="KQ1" s="1" t="n"/>
+      <c r="KR1" s="1" t="n"/>
+      <c r="KS1" s="1" t="n"/>
+      <c r="KT1" s="1" t="n"/>
+      <c r="KU1" s="1" t="n"/>
+      <c r="KV1" s="1" t="n"/>
+      <c r="KW1" s="1" t="n"/>
+      <c r="KX1" s="1" t="n"/>
+      <c r="KY1" s="1" t="n"/>
+      <c r="KZ1" s="1" t="n"/>
+      <c r="LA1" s="1" t="n"/>
+      <c r="LB1" s="1" t="n"/>
+      <c r="LC1" s="1" t="n"/>
+      <c r="LD1" s="1" t="n"/>
+      <c r="LE1" s="1" t="n"/>
+      <c r="LF1" s="1" t="n"/>
+      <c r="LG1" s="1" t="n"/>
+      <c r="LH1" s="1" t="n"/>
+      <c r="LI1" s="1" t="n"/>
+      <c r="LJ1" s="1" t="n"/>
+      <c r="LK1" s="1" t="n"/>
+      <c r="LL1" s="1" t="n"/>
+      <c r="LM1" s="1" t="n"/>
+      <c r="LN1" s="1" t="n"/>
+      <c r="LO1" s="1" t="n"/>
+      <c r="LP1" s="1" t="n"/>
+      <c r="LQ1" s="1" t="n"/>
+      <c r="LR1" s="1" t="n"/>
+      <c r="LS1" s="1" t="n"/>
+      <c r="LT1" s="1" t="n"/>
+      <c r="LU1" s="1" t="n"/>
+      <c r="LV1" s="1" t="n"/>
+      <c r="LW1" s="1" t="n"/>
+      <c r="LX1" s="1" t="n"/>
+      <c r="LY1" s="1" t="n"/>
+      <c r="LZ1" s="1" t="n"/>
+      <c r="MA1" s="1" t="n"/>
+      <c r="MB1" s="1" t="n"/>
+      <c r="MC1" s="1" t="n"/>
+      <c r="MD1" s="1" t="n"/>
+      <c r="ME1" s="1" t="n"/>
+      <c r="MF1" s="1" t="n"/>
+      <c r="MG1" s="1" t="n"/>
+      <c r="MH1" s="1" t="n"/>
+      <c r="MI1" s="1" t="n"/>
+      <c r="MJ1" s="1" t="n"/>
+      <c r="MK1" s="1" t="n"/>
+      <c r="ML1" s="1" t="n"/>
+      <c r="MM1" s="1" t="n"/>
+      <c r="MN1" s="1" t="n"/>
+      <c r="MO1" s="1" t="n"/>
+      <c r="MP1" s="1" t="n"/>
+      <c r="MQ1" s="1" t="n"/>
+      <c r="MR1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -870,7 +1182,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Fri 13</t>
+          <t>Sun 15</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -886,7 +1198,7 @@
       <c r="M2" s="1" t="n"/>
       <c r="N2" s="1" t="inlineStr">
         <is>
-          <t>Sat 14</t>
+          <t>Mon 16</t>
         </is>
       </c>
       <c r="O2" s="1" t="n"/>
@@ -903,7 +1215,7 @@
       <c r="Z2" s="1" t="n"/>
       <c r="AA2" s="1" t="inlineStr">
         <is>
-          <t>Sun 15</t>
+          <t>Tue 17</t>
         </is>
       </c>
       <c r="AB2" s="1" t="n"/>
@@ -920,7 +1232,7 @@
       <c r="AM2" s="1" t="n"/>
       <c r="AN2" s="1" t="inlineStr">
         <is>
-          <t>Mon 16</t>
+          <t>Wed 18</t>
         </is>
       </c>
       <c r="AO2" s="1" t="n"/>
@@ -937,7 +1249,7 @@
       <c r="AZ2" s="1" t="n"/>
       <c r="BA2" s="1" t="inlineStr">
         <is>
-          <t>Tue 17</t>
+          <t>Thu 19</t>
         </is>
       </c>
       <c r="BB2" s="1" t="n"/>
@@ -954,7 +1266,7 @@
       <c r="BM2" s="1" t="n"/>
       <c r="BN2" s="1" t="inlineStr">
         <is>
-          <t>Wed 18</t>
+          <t>Fri 20</t>
         </is>
       </c>
       <c r="BO2" s="1" t="n"/>
@@ -971,7 +1283,7 @@
       <c r="BZ2" s="1" t="n"/>
       <c r="CA2" s="1" t="inlineStr">
         <is>
-          <t>Thu 19</t>
+          <t>Sat 21</t>
         </is>
       </c>
       <c r="CB2" s="1" t="n"/>
@@ -988,7 +1300,7 @@
       <c r="CM2" s="1" t="n"/>
       <c r="CN2" s="1" t="inlineStr">
         <is>
-          <t>Fri 20</t>
+          <t>Sun 22</t>
         </is>
       </c>
       <c r="CO2" s="1" t="n"/>
@@ -1005,7 +1317,7 @@
       <c r="CZ2" s="1" t="n"/>
       <c r="DA2" s="1" t="inlineStr">
         <is>
-          <t>Sat 21</t>
+          <t>Mon 23</t>
         </is>
       </c>
       <c r="DB2" s="1" t="n"/>
@@ -1022,7 +1334,7 @@
       <c r="DM2" s="1" t="n"/>
       <c r="DN2" s="1" t="inlineStr">
         <is>
-          <t>Sun 22</t>
+          <t>Tue 24</t>
         </is>
       </c>
       <c r="DO2" s="1" t="n"/>
@@ -1039,7 +1351,7 @@
       <c r="DZ2" s="1" t="n"/>
       <c r="EA2" s="1" t="inlineStr">
         <is>
-          <t>Mon 23</t>
+          <t>Wed 25</t>
         </is>
       </c>
       <c r="EB2" s="1" t="n"/>
@@ -1056,7 +1368,7 @@
       <c r="EM2" s="1" t="n"/>
       <c r="EN2" s="1" t="inlineStr">
         <is>
-          <t>Tue 24</t>
+          <t>Thu 26</t>
         </is>
       </c>
       <c r="EO2" s="1" t="n"/>
@@ -1073,7 +1385,7 @@
       <c r="EZ2" s="1" t="n"/>
       <c r="FA2" s="1" t="inlineStr">
         <is>
-          <t>Wed 25</t>
+          <t>Fri 27</t>
         </is>
       </c>
       <c r="FB2" s="1" t="n"/>
@@ -1090,7 +1402,7 @@
       <c r="FM2" s="1" t="n"/>
       <c r="FN2" s="1" t="inlineStr">
         <is>
-          <t>Thu 26</t>
+          <t>Sat 28</t>
         </is>
       </c>
       <c r="FO2" s="1" t="n"/>
@@ -1107,7 +1419,7 @@
       <c r="FZ2" s="1" t="n"/>
       <c r="GA2" s="1" t="inlineStr">
         <is>
-          <t>Fri 27</t>
+          <t>Sun 01</t>
         </is>
       </c>
       <c r="GB2" s="1" t="n"/>
@@ -1124,7 +1436,7 @@
       <c r="GM2" s="1" t="n"/>
       <c r="GN2" s="1" t="inlineStr">
         <is>
-          <t>Sat 28</t>
+          <t>Mon 02</t>
         </is>
       </c>
       <c r="GO2" s="1" t="n"/>
@@ -1133,6 +1445,208 @@
       <c r="GR2" s="1" t="n"/>
       <c r="GS2" s="1" t="n"/>
       <c r="GT2" s="1" t="n"/>
+      <c r="GU2" s="1" t="n"/>
+      <c r="GV2" s="1" t="n"/>
+      <c r="GW2" s="1" t="n"/>
+      <c r="GX2" s="1" t="n"/>
+      <c r="GY2" s="1" t="n"/>
+      <c r="GZ2" s="1" t="n"/>
+      <c r="HA2" s="1" t="inlineStr">
+        <is>
+          <t>Tue 03</t>
+        </is>
+      </c>
+      <c r="HB2" s="1" t="n"/>
+      <c r="HC2" s="1" t="n"/>
+      <c r="HD2" s="1" t="n"/>
+      <c r="HE2" s="1" t="n"/>
+      <c r="HF2" s="1" t="n"/>
+      <c r="HG2" s="1" t="n"/>
+      <c r="HH2" s="1" t="n"/>
+      <c r="HI2" s="1" t="n"/>
+      <c r="HJ2" s="1" t="n"/>
+      <c r="HK2" s="1" t="n"/>
+      <c r="HL2" s="1" t="n"/>
+      <c r="HM2" s="1" t="n"/>
+      <c r="HN2" s="1" t="inlineStr">
+        <is>
+          <t>Wed 04</t>
+        </is>
+      </c>
+      <c r="HO2" s="1" t="n"/>
+      <c r="HP2" s="1" t="n"/>
+      <c r="HQ2" s="1" t="n"/>
+      <c r="HR2" s="1" t="n"/>
+      <c r="HS2" s="1" t="n"/>
+      <c r="HT2" s="1" t="n"/>
+      <c r="HU2" s="1" t="n"/>
+      <c r="HV2" s="1" t="n"/>
+      <c r="HW2" s="1" t="n"/>
+      <c r="HX2" s="1" t="n"/>
+      <c r="HY2" s="1" t="n"/>
+      <c r="HZ2" s="1" t="n"/>
+      <c r="IA2" s="1" t="inlineStr">
+        <is>
+          <t>Thu 05</t>
+        </is>
+      </c>
+      <c r="IB2" s="1" t="n"/>
+      <c r="IC2" s="1" t="n"/>
+      <c r="ID2" s="1" t="n"/>
+      <c r="IE2" s="1" t="n"/>
+      <c r="IF2" s="1" t="n"/>
+      <c r="IG2" s="1" t="n"/>
+      <c r="IH2" s="1" t="n"/>
+      <c r="II2" s="1" t="n"/>
+      <c r="IJ2" s="1" t="n"/>
+      <c r="IK2" s="1" t="n"/>
+      <c r="IL2" s="1" t="n"/>
+      <c r="IM2" s="1" t="n"/>
+      <c r="IN2" s="1" t="inlineStr">
+        <is>
+          <t>Fri 06</t>
+        </is>
+      </c>
+      <c r="IO2" s="1" t="n"/>
+      <c r="IP2" s="1" t="n"/>
+      <c r="IQ2" s="1" t="n"/>
+      <c r="IR2" s="1" t="n"/>
+      <c r="IS2" s="1" t="n"/>
+      <c r="IT2" s="1" t="n"/>
+      <c r="IU2" s="1" t="n"/>
+      <c r="IV2" s="1" t="n"/>
+      <c r="IW2" s="1" t="n"/>
+      <c r="IX2" s="1" t="n"/>
+      <c r="IY2" s="1" t="n"/>
+      <c r="IZ2" s="1" t="n"/>
+      <c r="JA2" s="1" t="inlineStr">
+        <is>
+          <t>Sat 07</t>
+        </is>
+      </c>
+      <c r="JB2" s="1" t="n"/>
+      <c r="JC2" s="1" t="n"/>
+      <c r="JD2" s="1" t="n"/>
+      <c r="JE2" s="1" t="n"/>
+      <c r="JF2" s="1" t="n"/>
+      <c r="JG2" s="1" t="n"/>
+      <c r="JH2" s="1" t="n"/>
+      <c r="JI2" s="1" t="n"/>
+      <c r="JJ2" s="1" t="n"/>
+      <c r="JK2" s="1" t="n"/>
+      <c r="JL2" s="1" t="n"/>
+      <c r="JM2" s="1" t="n"/>
+      <c r="JN2" s="1" t="inlineStr">
+        <is>
+          <t>Sun 08</t>
+        </is>
+      </c>
+      <c r="JO2" s="1" t="n"/>
+      <c r="JP2" s="1" t="n"/>
+      <c r="JQ2" s="1" t="n"/>
+      <c r="JR2" s="1" t="n"/>
+      <c r="JS2" s="1" t="n"/>
+      <c r="JT2" s="1" t="n"/>
+      <c r="JU2" s="1" t="n"/>
+      <c r="JV2" s="1" t="n"/>
+      <c r="JW2" s="1" t="n"/>
+      <c r="JX2" s="1" t="n"/>
+      <c r="JY2" s="1" t="n"/>
+      <c r="JZ2" s="1" t="n"/>
+      <c r="KA2" s="1" t="inlineStr">
+        <is>
+          <t>Mon 09</t>
+        </is>
+      </c>
+      <c r="KB2" s="1" t="n"/>
+      <c r="KC2" s="1" t="n"/>
+      <c r="KD2" s="1" t="n"/>
+      <c r="KE2" s="1" t="n"/>
+      <c r="KF2" s="1" t="n"/>
+      <c r="KG2" s="1" t="n"/>
+      <c r="KH2" s="1" t="n"/>
+      <c r="KI2" s="1" t="n"/>
+      <c r="KJ2" s="1" t="n"/>
+      <c r="KK2" s="1" t="n"/>
+      <c r="KL2" s="1" t="n"/>
+      <c r="KM2" s="1" t="n"/>
+      <c r="KN2" s="1" t="inlineStr">
+        <is>
+          <t>Tue 10</t>
+        </is>
+      </c>
+      <c r="KO2" s="1" t="n"/>
+      <c r="KP2" s="1" t="n"/>
+      <c r="KQ2" s="1" t="n"/>
+      <c r="KR2" s="1" t="n"/>
+      <c r="KS2" s="1" t="n"/>
+      <c r="KT2" s="1" t="n"/>
+      <c r="KU2" s="1" t="n"/>
+      <c r="KV2" s="1" t="n"/>
+      <c r="KW2" s="1" t="n"/>
+      <c r="KX2" s="1" t="n"/>
+      <c r="KY2" s="1" t="n"/>
+      <c r="KZ2" s="1" t="n"/>
+      <c r="LA2" s="1" t="inlineStr">
+        <is>
+          <t>Wed 11</t>
+        </is>
+      </c>
+      <c r="LB2" s="1" t="n"/>
+      <c r="LC2" s="1" t="n"/>
+      <c r="LD2" s="1" t="n"/>
+      <c r="LE2" s="1" t="n"/>
+      <c r="LF2" s="1" t="n"/>
+      <c r="LG2" s="1" t="n"/>
+      <c r="LH2" s="1" t="n"/>
+      <c r="LI2" s="1" t="n"/>
+      <c r="LJ2" s="1" t="n"/>
+      <c r="LK2" s="1" t="n"/>
+      <c r="LL2" s="1" t="n"/>
+      <c r="LM2" s="1" t="n"/>
+      <c r="LN2" s="1" t="inlineStr">
+        <is>
+          <t>Thu 12</t>
+        </is>
+      </c>
+      <c r="LO2" s="1" t="n"/>
+      <c r="LP2" s="1" t="n"/>
+      <c r="LQ2" s="1" t="n"/>
+      <c r="LR2" s="1" t="n"/>
+      <c r="LS2" s="1" t="n"/>
+      <c r="LT2" s="1" t="n"/>
+      <c r="LU2" s="1" t="n"/>
+      <c r="LV2" s="1" t="n"/>
+      <c r="LW2" s="1" t="n"/>
+      <c r="LX2" s="1" t="n"/>
+      <c r="LY2" s="1" t="n"/>
+      <c r="LZ2" s="1" t="n"/>
+      <c r="MA2" s="1" t="inlineStr">
+        <is>
+          <t>Fri 13</t>
+        </is>
+      </c>
+      <c r="MB2" s="1" t="n"/>
+      <c r="MC2" s="1" t="n"/>
+      <c r="MD2" s="1" t="n"/>
+      <c r="ME2" s="1" t="n"/>
+      <c r="MF2" s="1" t="n"/>
+      <c r="MG2" s="1" t="n"/>
+      <c r="MH2" s="1" t="n"/>
+      <c r="MI2" s="1" t="n"/>
+      <c r="MJ2" s="1" t="n"/>
+      <c r="MK2" s="1" t="n"/>
+      <c r="ML2" s="1" t="n"/>
+      <c r="MM2" s="1" t="n"/>
+      <c r="MN2" s="1" t="inlineStr">
+        <is>
+          <t>Sat 14</t>
+        </is>
+      </c>
+      <c r="MO2" s="1" t="n"/>
+      <c r="MP2" s="1" t="n"/>
+      <c r="MQ2" s="1" t="n"/>
+      <c r="MR2" s="1" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -2135,8 +2649,778 @@
           <t>12</t>
         </is>
       </c>
-      <c r="GS3" s="1" t="n"/>
-      <c r="GT3" s="1" t="n"/>
+      <c r="GS3" s="1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="GT3" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="GU3" s="1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="GV3" s="1" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="GW3" s="1" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="GX3" s="1" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="GY3" s="1" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="GZ3" s="1" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="HA3" s="1" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="HB3" s="1" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="HC3" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="HD3" s="1" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="HE3" s="1" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="HF3" s="1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="HG3" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="HH3" s="1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="HI3" s="1" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="HJ3" s="1" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="HK3" s="1" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="HL3" s="1" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="HM3" s="1" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="HN3" s="1" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="HO3" s="1" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="HP3" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="HQ3" s="1" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="HR3" s="1" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="HS3" s="1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="HT3" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="HU3" s="1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="HV3" s="1" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="HW3" s="1" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="HX3" s="1" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="HY3" s="1" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="HZ3" s="1" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="IA3" s="1" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="IB3" s="1" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="IC3" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="ID3" s="1" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="IE3" s="1" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="IF3" s="1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="IG3" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="IH3" s="1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="II3" s="1" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="IJ3" s="1" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="IK3" s="1" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="IL3" s="1" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="IM3" s="1" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="IN3" s="1" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="IO3" s="1" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="IP3" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="IQ3" s="1" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="IR3" s="1" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="IS3" s="1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="IT3" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="IU3" s="1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="IV3" s="1" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="IW3" s="1" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="IX3" s="1" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="IY3" s="1" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="IZ3" s="1" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="JA3" s="1" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="JB3" s="1" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="JC3" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="JD3" s="1" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="JE3" s="1" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="JF3" s="1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="JG3" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="JH3" s="1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="JI3" s="1" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="JJ3" s="1" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="JK3" s="1" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="JL3" s="1" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="JM3" s="1" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="JN3" s="1" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="JO3" s="1" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="JP3" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="JQ3" s="1" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="JR3" s="1" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="JS3" s="1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="JT3" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="JU3" s="1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="JV3" s="1" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="JW3" s="1" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="JX3" s="1" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="JY3" s="1" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="JZ3" s="1" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="KA3" s="1" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="KB3" s="1" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="KC3" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="KD3" s="1" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="KE3" s="1" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="KF3" s="1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="KG3" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="KH3" s="1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="KI3" s="1" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="KJ3" s="1" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="KK3" s="1" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="KL3" s="1" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="KM3" s="1" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="KN3" s="1" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="KO3" s="1" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="KP3" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="KQ3" s="1" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="KR3" s="1" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="KS3" s="1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="KT3" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="KU3" s="1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="KV3" s="1" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="KW3" s="1" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="KX3" s="1" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="KY3" s="1" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="KZ3" s="1" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="LA3" s="1" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="LB3" s="1" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="LC3" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="LD3" s="1" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="LE3" s="1" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="LF3" s="1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="LG3" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="LH3" s="1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="LI3" s="1" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="LJ3" s="1" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="LK3" s="1" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="LL3" s="1" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="LM3" s="1" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="LN3" s="1" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="LO3" s="1" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="LP3" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="LQ3" s="1" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="LR3" s="1" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="LS3" s="1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="LT3" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="LU3" s="1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="LV3" s="1" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="LW3" s="1" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="LX3" s="1" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="LY3" s="1" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="LZ3" s="1" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="MA3" s="1" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="MB3" s="1" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="MC3" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="MD3" s="1" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="ME3" s="1" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="MF3" s="1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="MG3" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="MH3" s="1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="MI3" s="1" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="MJ3" s="1" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="MK3" s="1" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="ML3" s="1" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="MM3" s="1" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="MN3" s="1" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="MO3" s="1" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="MP3" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="MQ3" s="1" t="n"/>
+      <c r="MR3" s="1" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -2144,14 +3428,9 @@
           <t>Salle1</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Cours68 - Prof6</t>
-        </is>
-      </c>
-      <c r="EB4" s="2" t="inlineStr">
-        <is>
-          <t>Cours20 - Prof5</t>
+      <c r="HB4" s="2" t="inlineStr">
+        <is>
+          <t>Cours1 - Prof1</t>
         </is>
       </c>
     </row>
@@ -2161,26 +3440,26 @@
           <t>Salle10</t>
         </is>
       </c>
-      <c r="BB5" s="2" t="inlineStr">
-        <is>
-          <t>Cours149 - Prof4</t>
+      <c r="GO5" s="2" t="inlineStr">
+        <is>
+          <t>Cours8 - Prof1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Salle12</t>
-        </is>
-      </c>
-      <c r="AB6" s="2" t="inlineStr">
-        <is>
-          <t>Cours137 - Prof8</t>
-        </is>
-      </c>
-      <c r="DO6" s="2" t="inlineStr">
-        <is>
-          <t>Cours30 - Prof1</t>
+          <t>Salle13</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Cours42 - Prof17</t>
+        </is>
+      </c>
+      <c r="FO6" s="2" t="inlineStr">
+        <is>
+          <t>Cours32 - Prof8</t>
         </is>
       </c>
     </row>
@@ -2190,9 +3469,14 @@
           <t>Salle14</t>
         </is>
       </c>
-      <c r="AO7" s="2" t="inlineStr">
-        <is>
-          <t>Cours56 - Prof8</t>
+      <c r="JB7" s="2" t="inlineStr">
+        <is>
+          <t>Cours54 - Prof4</t>
+        </is>
+      </c>
+      <c r="JD7" s="2" t="inlineStr">
+        <is>
+          <t>Cours33 - Prof11</t>
         </is>
       </c>
     </row>
@@ -2202,412 +3486,143 @@
           <t>Salle15</t>
         </is>
       </c>
-      <c r="CB8" s="2" t="inlineStr">
-        <is>
-          <t>Cours96 - Prof5</t>
-        </is>
-      </c>
-      <c r="EO8" s="2" t="inlineStr">
-        <is>
-          <t>Cours102 - Prof8</t>
-        </is>
-      </c>
-      <c r="FO8" s="2" t="inlineStr">
-        <is>
-          <t>Cours135 - Prof5</t>
+      <c r="DB8" s="2" t="inlineStr">
+        <is>
+          <t>Cours36 - Prof7</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Salle16</t>
-        </is>
-      </c>
-      <c r="BO9" s="2" t="inlineStr">
-        <is>
-          <t>Cours52 - Prof4</t>
+          <t>Salle18</t>
+        </is>
+      </c>
+      <c r="MO9" s="2" t="inlineStr">
+        <is>
+          <t>Cours49 - Prof9</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Salle17</t>
-        </is>
-      </c>
-      <c r="AO10" s="2" t="inlineStr">
-        <is>
-          <t>Cours3 - Prof9</t>
+          <t>Salle22</t>
         </is>
       </c>
       <c r="BO10" s="2" t="inlineStr">
         <is>
-          <t>Cours156 - Prof10</t>
-        </is>
-      </c>
-      <c r="EB10" s="2" t="inlineStr">
-        <is>
-          <t>Cours159 - Prof1</t>
-        </is>
-      </c>
-      <c r="EO10" s="2" t="inlineStr">
-        <is>
-          <t>Cours160 - Prof1</t>
+          <t>Cours4 - Prof12</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Salle18</t>
-        </is>
-      </c>
-      <c r="DB11" s="2" t="inlineStr">
-        <is>
-          <t>Cours26 - Prof6</t>
-        </is>
-      </c>
-      <c r="DC11" s="2" t="inlineStr">
-        <is>
-          <t>Cours39 - Prof3</t>
-        </is>
-      </c>
-      <c r="FB11" s="2" t="inlineStr">
-        <is>
-          <t>Cours65 - Prof1</t>
+          <t>Salle23</t>
+        </is>
+      </c>
+      <c r="GO11" s="2" t="inlineStr">
+        <is>
+          <t>Cours20 - Prof12</t>
+        </is>
+      </c>
+      <c r="HB11" s="2" t="inlineStr">
+        <is>
+          <t>Cours34 - Prof9</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>Salle19</t>
-        </is>
-      </c>
-      <c r="BO12" s="2" t="inlineStr">
-        <is>
-          <t>Cours130 - Prof2</t>
-        </is>
-      </c>
-      <c r="CO12" s="2" t="inlineStr">
-        <is>
-          <t>Cours163 - Prof3</t>
+          <t>Salle30</t>
+        </is>
+      </c>
+      <c r="FO12" s="2" t="inlineStr">
+        <is>
+          <t>Cours40 - Prof19</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Salle2</t>
-        </is>
-      </c>
-      <c r="AO13" s="2" t="inlineStr">
-        <is>
-          <t>Cours16 - Prof4</t>
-        </is>
-      </c>
-      <c r="FB13" s="2" t="inlineStr">
-        <is>
-          <t>Cours22 - Prof6</t>
-        </is>
-      </c>
-      <c r="GO13" s="2" t="inlineStr">
-        <is>
-          <t>Cours114 - Prof10</t>
+          <t>Salle6</t>
+        </is>
+      </c>
+      <c r="CB13" s="2" t="inlineStr">
+        <is>
+          <t>Cours57 - Prof5</t>
+        </is>
+      </c>
+      <c r="EB13" s="2" t="inlineStr">
+        <is>
+          <t>Cours25 - Prof5</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>Salle20</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>Cours5 - Prof8</t>
-        </is>
-      </c>
-      <c r="AO14" s="2" t="inlineStr">
-        <is>
-          <t>Cours78 - Prof6</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>Salle21</t>
-        </is>
-      </c>
-      <c r="EO15" s="2" t="inlineStr">
-        <is>
-          <t>Cours131 - Prof6</t>
-        </is>
-      </c>
-      <c r="GB15" s="2" t="inlineStr">
-        <is>
-          <t>Cours144 - Prof2</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>Salle22</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Cours97 - Prof7</t>
-        </is>
-      </c>
-      <c r="DB16" s="2" t="inlineStr">
-        <is>
-          <t>Cours94 - Prof4</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>Salle23</t>
-        </is>
-      </c>
-      <c r="BB17" s="2" t="inlineStr">
-        <is>
-          <t>Cours115 - Prof2</t>
-        </is>
-      </c>
-      <c r="BO17" s="2" t="inlineStr">
-        <is>
-          <t>Cours133 - Prof7</t>
-        </is>
-      </c>
-      <c r="GO17" s="2" t="inlineStr">
-        <is>
-          <t>Cours136 - Prof7</t>
-        </is>
-      </c>
-      <c r="GR17" s="2" t="inlineStr">
-        <is>
-          <t>Cours118 - Prof10</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>Salle24</t>
-        </is>
-      </c>
-      <c r="BO18" s="2" t="inlineStr">
-        <is>
-          <t>Cours6 - Prof6</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>Salle26</t>
-        </is>
-      </c>
-      <c r="DO19" s="2" t="inlineStr">
-        <is>
-          <t>Cours125 - Prof9</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>Salle27</t>
-        </is>
-      </c>
-      <c r="EO20" s="2" t="inlineStr">
-        <is>
-          <t>Cours98 - Prof2</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>Salle30</t>
-        </is>
-      </c>
-      <c r="DB21" s="2" t="inlineStr">
-        <is>
-          <t>Cours122 - Prof2</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>Salle4</t>
-        </is>
-      </c>
-      <c r="FO22" s="2" t="inlineStr">
-        <is>
-          <t>Cours64 - Prof10</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>Salle5</t>
-        </is>
-      </c>
-      <c r="GB23" s="2" t="inlineStr">
-        <is>
-          <t>Cours158 - Prof6</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>Salle6</t>
-        </is>
-      </c>
-      <c r="AO24" s="2" t="inlineStr">
-        <is>
-          <t>Cours44 - Prof1</t>
-        </is>
-      </c>
-      <c r="DO24" s="2" t="inlineStr">
-        <is>
-          <t>Cours55 - Prof5</t>
-        </is>
-      </c>
-      <c r="FB24" s="2" t="inlineStr">
-        <is>
-          <t>Cours143 - Prof9</t>
-        </is>
-      </c>
-      <c r="GB24" s="2" t="inlineStr">
-        <is>
-          <t>Cours85 - Prof9</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>Salle7</t>
-        </is>
-      </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>Cours53 - Prof10</t>
-        </is>
-      </c>
-      <c r="BB25" s="2" t="inlineStr">
-        <is>
-          <t>Cours129 - Prof8</t>
-        </is>
-      </c>
-      <c r="BE25" s="2" t="inlineStr">
-        <is>
-          <t>Cours128 - Prof2</t>
-        </is>
-      </c>
-      <c r="GO25" s="2" t="inlineStr">
-        <is>
-          <t>Cours75 - Prof9</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>Salle9</t>
-        </is>
-      </c>
-      <c r="AO26" s="2" t="inlineStr">
-        <is>
-          <t>Cours74 - Prof7</t>
-        </is>
-      </c>
-      <c r="CO26" s="2" t="inlineStr">
-        <is>
-          <t>Cours37 - Prof9</t>
+          <t>Salle8</t>
+        </is>
+      </c>
+      <c r="BB14" s="2" t="inlineStr">
+        <is>
+          <t>Cours44 - Prof19</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="67">
+  <mergeCells count="47">
     <mergeCell ref="B2:M2"/>
-    <mergeCell ref="DB21"/>
     <mergeCell ref="AN2:AZ2"/>
-    <mergeCell ref="CO26"/>
-    <mergeCell ref="DO6"/>
-    <mergeCell ref="BO9:BP9"/>
-    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="LN2:LZ2"/>
+    <mergeCell ref="MO9:MP9"/>
     <mergeCell ref="DA2:DM2"/>
-    <mergeCell ref="GB24:GC24"/>
-    <mergeCell ref="BB5:BD5"/>
+    <mergeCell ref="MN2:MP2"/>
     <mergeCell ref="FA2:FM2"/>
-    <mergeCell ref="DO24"/>
-    <mergeCell ref="FO22:FR22"/>
-    <mergeCell ref="DB16:DD16"/>
-    <mergeCell ref="BB17"/>
+    <mergeCell ref="FO12:FP12"/>
     <mergeCell ref="AA2:AM2"/>
-    <mergeCell ref="EO20:EP20"/>
-    <mergeCell ref="DO19:DQ19"/>
-    <mergeCell ref="GB23:GC23"/>
-    <mergeCell ref="GR17"/>
-    <mergeCell ref="CB8:CD8"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="GO17:GQ17"/>
-    <mergeCell ref="AO10:AQ10"/>
-    <mergeCell ref="BB25:BD25"/>
+    <mergeCell ref="GN2:GZ2"/>
+    <mergeCell ref="DB8:DE8"/>
+    <mergeCell ref="IN2:IZ2"/>
+    <mergeCell ref="HB11"/>
+    <mergeCell ref="JB7:JC7"/>
+    <mergeCell ref="HB4:HC4"/>
+    <mergeCell ref="LA2:LM2"/>
+    <mergeCell ref="BO10"/>
+    <mergeCell ref="GO5:GQ5"/>
+    <mergeCell ref="EB13:EC13"/>
     <mergeCell ref="BN2:BZ2"/>
     <mergeCell ref="DN2:DZ2"/>
-    <mergeCell ref="EO15:ER15"/>
-    <mergeCell ref="BO18:BQ18"/>
     <mergeCell ref="GA2:GM2"/>
-    <mergeCell ref="AO7:AR7"/>
-    <mergeCell ref="FB24:FD24"/>
+    <mergeCell ref="FO6:FQ6"/>
+    <mergeCell ref="IA2:IM2"/>
+    <mergeCell ref="BB14:BC14"/>
+    <mergeCell ref="HN2:HZ2"/>
+    <mergeCell ref="JD7:JF7"/>
+    <mergeCell ref="JN2:JZ2"/>
     <mergeCell ref="BA2:BM2"/>
-    <mergeCell ref="DC11"/>
-    <mergeCell ref="CO12:CQ12"/>
-    <mergeCell ref="GS2:GT2"/>
+    <mergeCell ref="MA2:MM2"/>
+    <mergeCell ref="GO11:GR11"/>
     <mergeCell ref="CN2:CZ2"/>
-    <mergeCell ref="EO10:ER10"/>
     <mergeCell ref="EN2:EZ2"/>
-    <mergeCell ref="BO12:BP12"/>
-    <mergeCell ref="FB13:FC13"/>
-    <mergeCell ref="FB11:FE11"/>
-    <mergeCell ref="GS1"/>
-    <mergeCell ref="EB10"/>
-    <mergeCell ref="BO17:BR17"/>
-    <mergeCell ref="GO13:GP13"/>
-    <mergeCell ref="AB6:AD6"/>
-    <mergeCell ref="AO26:AP26"/>
+    <mergeCell ref="HA2:HM2"/>
+    <mergeCell ref="JA2:JM2"/>
     <mergeCell ref="N2:Z2"/>
-    <mergeCell ref="FO8:FR8"/>
-    <mergeCell ref="EB4:ED4"/>
-    <mergeCell ref="BE25:BH25"/>
-    <mergeCell ref="AO24:AR24"/>
-    <mergeCell ref="DB11"/>
-    <mergeCell ref="GO25:GR25"/>
+    <mergeCell ref="MQ2:MR2"/>
+    <mergeCell ref="B1:FZ1"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="CB13:CC13"/>
+    <mergeCell ref="KN2:KZ2"/>
+    <mergeCell ref="MQ1"/>
     <mergeCell ref="CA2:CM2"/>
-    <mergeCell ref="GN2:GR2"/>
-    <mergeCell ref="AO14"/>
     <mergeCell ref="EA2:EM2"/>
-    <mergeCell ref="O25"/>
-    <mergeCell ref="B1:GR1"/>
-    <mergeCell ref="O14:P14"/>
-    <mergeCell ref="GB15:GE15"/>
+    <mergeCell ref="GA1:MP1"/>
     <mergeCell ref="FN2:FZ2"/>
-    <mergeCell ref="BO10:BP10"/>
-    <mergeCell ref="AO13:AQ13"/>
-    <mergeCell ref="EO8:ER8"/>
+    <mergeCell ref="KA2:KM2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2619,7 +3634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2664,1345 +3679,421 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46074.375</v>
+        <v>46076.375</v>
       </c>
       <c r="B2" s="4" t="n">
-        <v>46074.41666666666</v>
+        <v>46076.54166666666</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Salle18</t>
+          <t>Salle15</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Cours26</t>
+          <t>Cours36</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Prof6</t>
+          <t>Prof7</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Prof6</t>
+          <t>Prof7</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46071.375</v>
+        <v>46074.375</v>
       </c>
       <c r="B3" s="4" t="n">
-        <v>46071.45833333334</v>
+        <v>46074.45833333334</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Salle19</t>
+          <t>Salle6</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Cours130</t>
+          <t>Cours57</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Prof2</t>
+          <t>Prof5</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Prof2</t>
+          <t>Prof5</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46073.375</v>
+        <v>46078.375</v>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46073.41666666666</v>
+        <v>46078.45833333334</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Salle9</t>
+          <t>Salle6</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Cours37</t>
+          <t>Cours25</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Prof9</t>
+          <t>Prof5</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Prof9</t>
+          <t>Prof5</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46071.375</v>
+        <v>46081.375</v>
       </c>
       <c r="B5" s="4" t="n">
-        <v>46071.45833333334</v>
+        <v>46081.5</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Salle17</t>
+          <t>Salle13</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Cours156</t>
+          <t>Cours32</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Prof10</t>
+          <t>Prof8</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Prof10</t>
+          <t>Prof8</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46080.375</v>
+        <v>46081.375</v>
       </c>
       <c r="B6" s="4" t="n">
-        <v>46080.45833333334</v>
+        <v>46081.45833333334</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Salle5</t>
+          <t>Salle30</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Cours158</t>
+          <t>Cours40</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Prof6</t>
+          <t>Prof19</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Prof6</t>
+          <t>Prof19</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46069.375</v>
+        <v>46068.375</v>
       </c>
       <c r="B7" s="4" t="n">
-        <v>46069.45833333334</v>
+        <v>46068.45833333334</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Salle9</t>
+          <t>Salle13</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Cours74</t>
+          <t>Cours42</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Prof7</t>
+          <t>Prof17</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Prof7</t>
+          <t>Prof17</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46066.375</v>
+        <v>46083.375</v>
       </c>
       <c r="B8" s="4" t="n">
-        <v>46066.54166666666</v>
+        <v>46083.5</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Salle1</t>
+          <t>Salle10</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Cours68</t>
+          <t>Cours8</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Prof6</t>
+          <t>Prof1</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Prof6</t>
+          <t>Prof1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46077.375</v>
+        <v>46084.375</v>
       </c>
       <c r="B9" s="4" t="n">
-        <v>46077.54166666666</v>
+        <v>46084.41666666666</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Salle17</t>
+          <t>Salle23</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Cours160</t>
+          <t>Cours34</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Prof1</t>
+          <t>Prof9</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Prof1</t>
+          <t>Prof9</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46081.375</v>
+        <v>46083.375</v>
       </c>
       <c r="B10" s="4" t="n">
-        <v>46081.54166666666</v>
+        <v>46083.54166666666</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Salle7</t>
+          <t>Salle23</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Cours75</t>
+          <t>Cours20</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Prof9</t>
+          <t>Prof12</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Prof9</t>
+          <t>Prof12</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46068.375</v>
+        <v>46095.375</v>
       </c>
       <c r="B11" s="4" t="n">
-        <v>46068.5</v>
+        <v>46095.45833333334</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Salle12</t>
+          <t>Salle18</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Cours137</t>
+          <t>Cours49</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Prof8</t>
+          <t>Prof9</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Prof8</t>
+          <t>Prof9</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46071.375</v>
+        <v>46088.375</v>
       </c>
       <c r="B12" s="4" t="n">
-        <v>46071.5</v>
+        <v>46088.45833333334</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Salle24</t>
+          <t>Salle14</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Cours6</t>
+          <t>Cours54</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Prof6</t>
+          <t>Prof4</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Prof6</t>
+          <t>Prof4</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46081.375</v>
+        <v>46088.45833333334</v>
       </c>
       <c r="B13" s="4" t="n">
-        <v>46081.5</v>
+        <v>46088.58333333334</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Salle23</t>
+          <t>Salle14</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Cours136</t>
+          <t>Cours33</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Prof7</t>
+          <t>Prof11</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Prof7</t>
+          <t>Prof11</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46079.375</v>
+        <v>46072.375</v>
       </c>
       <c r="B14" s="4" t="n">
-        <v>46079.54166666666</v>
+        <v>46072.45833333334</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Salle15</t>
+          <t>Salle8</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Cours135</t>
+          <t>Cours44</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Prof5</t>
+          <t>Prof19</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Prof5</t>
+          <t>Prof19</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46078.375</v>
+        <v>46073.375</v>
       </c>
       <c r="B15" s="4" t="n">
-        <v>46078.5</v>
+        <v>46073.41666666666</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Salle6</t>
+          <t>Salle22</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Cours143</t>
+          <t>Cours4</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Prof9</t>
+          <t>Prof12</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Prof9</t>
+          <t>Prof12</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46067.375</v>
+        <v>46084.375</v>
       </c>
       <c r="B16" s="4" t="n">
-        <v>46067.41666666666</v>
+        <v>46084.45833333334</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Salle7</t>
+          <t>Salle1</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Cours53</t>
+          <t>Cours1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Prof10</t>
+          <t>Prof1</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Prof10</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n">
-        <v>46071.375</v>
-      </c>
-      <c r="B17" s="4" t="n">
-        <v>46071.45833333334</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Salle16</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Cours52</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Prof4</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Prof4</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n">
-        <v>46073.375</v>
-      </c>
-      <c r="B18" s="4" t="n">
-        <v>46073.5</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Salle19</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Cours163</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Prof3</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Prof3</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n">
-        <v>46074.375</v>
-      </c>
-      <c r="B19" s="4" t="n">
-        <v>46074.41666666666</v>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Salle30</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Cours122</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Prof2</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Prof2</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
-        <v>46070.375</v>
-      </c>
-      <c r="B20" s="4" t="n">
-        <v>46070.41666666666</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Salle23</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Cours115</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Prof2</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Prof2</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="n">
-        <v>46069.375</v>
-      </c>
-      <c r="B21" s="4" t="n">
-        <v>46069.5</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Salle17</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Cours3</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Prof9</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Prof9</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="n">
-        <v>46069.375</v>
-      </c>
-      <c r="B22" s="4" t="n">
-        <v>46069.54166666666</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Salle14</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Cours56</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Prof8</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Prof8</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="n">
-        <v>46074.375</v>
-      </c>
-      <c r="B23" s="4" t="n">
-        <v>46074.5</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Salle22</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Cours94</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Prof4</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Prof4</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="n">
-        <v>46075.375</v>
-      </c>
-      <c r="B24" s="4" t="n">
-        <v>46075.41666666666</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Salle12</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Cours30</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
           <t>Prof1</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Prof1</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="n">
-        <v>46078.375</v>
-      </c>
-      <c r="B25" s="4" t="n">
-        <v>46078.54166666666</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Salle18</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Cours65</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Prof1</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Prof1</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="n">
-        <v>46066.375</v>
-      </c>
-      <c r="B26" s="4" t="n">
-        <v>46066.45833333334</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Salle22</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Cours97</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Prof7</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Prof7</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="n">
-        <v>46070.375</v>
-      </c>
-      <c r="B27" s="4" t="n">
-        <v>46070.5</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Salle10</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Cours149</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Prof4</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Prof4</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="n">
-        <v>46081.5</v>
-      </c>
-      <c r="B28" s="4" t="n">
-        <v>46081.54166666666</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Salle23</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Cours118</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Prof10</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Prof10</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="n">
-        <v>46077.375</v>
-      </c>
-      <c r="B29" s="4" t="n">
-        <v>46077.45833333334</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Salle27</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Cours98</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Prof2</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Prof2</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="n">
-        <v>46069.375</v>
-      </c>
-      <c r="B30" s="4" t="n">
-        <v>46069.5</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Salle2</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Cours16</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Prof4</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Prof4</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="n">
-        <v>46076.375</v>
-      </c>
-      <c r="B31" s="4" t="n">
-        <v>46076.41666666666</v>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Salle17</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Cours159</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Prof1</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Prof1</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="n">
-        <v>46077.375</v>
-      </c>
-      <c r="B32" s="4" t="n">
-        <v>46077.54166666666</v>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Salle15</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Cours102</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Prof8</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Prof8</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="n">
-        <v>46080.375</v>
-      </c>
-      <c r="B33" s="4" t="n">
-        <v>46080.54166666666</v>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Salle21</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Cours144</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Prof2</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Prof2</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="n">
-        <v>46077.375</v>
-      </c>
-      <c r="B34" s="4" t="n">
-        <v>46077.54166666666</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Salle21</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Cours131</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Prof6</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Prof6</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="n">
-        <v>46080.375</v>
-      </c>
-      <c r="B35" s="4" t="n">
-        <v>46080.45833333334</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Salle6</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Cours85</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Prof9</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Prof9</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="n">
-        <v>46069.375</v>
-      </c>
-      <c r="B36" s="4" t="n">
-        <v>46069.54166666666</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Salle6</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Cours44</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Prof1</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Prof1</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="n">
-        <v>46069.375</v>
-      </c>
-      <c r="B37" s="4" t="n">
-        <v>46069.41666666666</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Salle20</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Cours78</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Prof6</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Prof6</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="n">
-        <v>46075.375</v>
-      </c>
-      <c r="B38" s="4" t="n">
-        <v>46075.41666666666</v>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Salle6</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Cours55</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Prof5</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>Prof5</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="n">
-        <v>46079.375</v>
-      </c>
-      <c r="B39" s="4" t="n">
-        <v>46079.54166666666</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Salle4</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Cours64</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Prof10</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Prof10</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="n">
-        <v>46071.375</v>
-      </c>
-      <c r="B40" s="4" t="n">
-        <v>46071.54166666666</v>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Salle23</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Cours133</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Prof7</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Prof7</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="n">
-        <v>46078.375</v>
-      </c>
-      <c r="B41" s="4" t="n">
-        <v>46078.45833333334</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Salle2</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Cours22</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Prof6</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Prof6</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="n">
-        <v>46076.375</v>
-      </c>
-      <c r="B42" s="4" t="n">
-        <v>46076.5</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Salle1</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Cours20</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Prof5</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Prof5</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="n">
-        <v>46074.41666666666</v>
-      </c>
-      <c r="B43" s="4" t="n">
-        <v>46074.45833333334</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Salle18</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Cours39</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Prof3</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Prof3</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="n">
-        <v>46067.375</v>
-      </c>
-      <c r="B44" s="4" t="n">
-        <v>46067.45833333334</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Salle20</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Cours5</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Prof8</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Prof8</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="n">
-        <v>46075.375</v>
-      </c>
-      <c r="B45" s="4" t="n">
-        <v>46075.5</v>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Salle26</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Cours125</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Prof9</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Prof9</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="n">
-        <v>46070.375</v>
-      </c>
-      <c r="B46" s="4" t="n">
-        <v>46070.5</v>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Salle7</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Cours129</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Prof8</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>Prof8</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="n">
-        <v>46081.375</v>
-      </c>
-      <c r="B47" s="4" t="n">
-        <v>46081.45833333334</v>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Salle2</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Cours114</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Prof10</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Prof10</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="n">
-        <v>46070.5</v>
-      </c>
-      <c r="B48" s="4" t="n">
-        <v>46070.66666666666</v>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Salle7</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Cours128</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Prof2</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>Prof2</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="n">
-        <v>46072.375</v>
-      </c>
-      <c r="B49" s="4" t="n">
-        <v>46072.5</v>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Salle15</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Cours96</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Prof5</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Prof5</t>
         </is>
       </c>
     </row>

</xml_diff>